<commit_message>
I don't know the change
</commit_message>
<xml_diff>
--- a/log/theme_resources.xlsx
+++ b/log/theme_resources.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Gamemaker\2026-China\Architects\log\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{664FBC8F-9FA6-4974-B3D7-195C824E63B4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{06CE339D-8312-4EC6-8171-179BFAF150A8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-23148" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -202,7 +202,7 @@
     <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
     </xf>
@@ -689,5 +689,6 @@
   </sheetData>
   <phoneticPr fontId="1" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>